<commit_message>
target renegade - up to level 1
</commit_message>
<xml_diff>
--- a/TargetRenegade/compare.xlsx
+++ b/TargetRenegade/compare.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\adelikat-tas\TargetRenegade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{286F5646-9AD4-4AEA-B7DC-BED976E7F124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD6C593-53F7-4897-9597-B2267CACD6C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="46920" yWindow="3825" windowWidth="10245" windowHeight="12285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="V2" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Place</t>
   </si>
@@ -43,6 +43,30 @@
   <si>
     <t>v1</t>
   </si>
+  <si>
+    <t>1st input</t>
+  </si>
+  <si>
+    <t>title screen appears</t>
+  </si>
+  <si>
+    <t>title screen disappears</t>
+  </si>
+  <si>
+    <t>start to begin appears</t>
+  </si>
+  <si>
+    <t>start to begin disappears</t>
+  </si>
+  <si>
+    <t>cut scene appears</t>
+  </si>
+  <si>
+    <t>cut scene disappears</t>
+  </si>
+  <si>
+    <t>lv 1 appears</t>
+  </si>
 </sst>
 </file>
 
@@ -51,12 +75,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00;[Red]&quot;-&quot;[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -154,25 +185,26 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="6" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="7">
@@ -519,51 +551,120 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D2" s="3" t="str">
+      <c r="A2" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="2">
+        <v>207</v>
+      </c>
+      <c r="C2" s="2">
+        <v>207</v>
+      </c>
+      <c r="D2" s="3">
         <f t="shared" ref="D2:D70" si="0">IF(C2&lt;&gt;"",IF(B2&lt;&gt;"",C2-B2,"-"), "-")</f>
-        <v>-</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D3" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A3" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2">
+        <v>690</v>
+      </c>
+      <c r="C3" s="2">
+        <v>690</v>
+      </c>
+      <c r="D3" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D4" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1102</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1102</v>
+      </c>
+      <c r="D4" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D5" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1140</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1140</v>
+      </c>
+      <c r="D5" s="3">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D6" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A6" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1170</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1179</v>
+      </c>
+      <c r="D6" s="3">
+        <f t="shared" si="0"/>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="2">
+        <v>1207</v>
+      </c>
       <c r="D7" s="3" t="str">
         <f t="shared" si="0"/>
         <v>-</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D8" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A8" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1324</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1396</v>
+      </c>
+      <c r="D8" s="3">
+        <f t="shared" si="0"/>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D9" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>-</v>
+      <c r="A9" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1354</v>
+      </c>
+      <c r="C9" s="2">
+        <v>1426</v>
+      </c>
+      <c r="D9" s="3">
+        <f t="shared" si="0"/>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1011,7 +1112,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="10" type="noConversion"/>
+  <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0" right="0" top="0.39410000000000006" bottom="0.39410000000000006" header="0" footer="0"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <headerFooter>

</xml_diff>